<commit_message>
Add import parsers for features, steps, and content sections
Wire three new parsers into the full super.money page import so the live
sections populate the new blocks with real content:
- supermoney-features: gathers the consecutive alternating image+text feature
  sections (cardsection / threerow / creditcard); first section becomes the
  block title/subtitle, the rest become feature rows.
- supermoney-steps: 'How to get started?' icon+text steps.
- supermoney-content: long-form SEO section with the fee/cashback tables,
  emitted as a single richtext cell (headings, lists, tables preserved).
- import-supermoney-full: register the parsers + selectors; rebuild bundle.

Verified in preview: header + hero + features + steps + content + footer all
render in order matching the live page.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-supermoney-full.report.xlsx
+++ b/tools/importer/reports/import-supermoney-full.report.xlsx
@@ -130,7 +130,7 @@
     <t>credit-cards/811-super-money-credit-card.report.json</t>
   </si>
   <si>
-    <t>["supermoney-header","supermoney-hero","supermoney-footer"]</t>
+    <t>["supermoney-header","supermoney-hero","supermoney-features","supermoney-features","supermoney-features","supermoney-features","supermoney-steps","supermoney-content","supermoney-footer"]</t>
   </si>
   <si>
     <t>credit-cards/811-super-money-credit-card</t>
@@ -139,7 +139,7 @@
     <t>supermoney-full</t>
   </si>
   <si>
-    <t>2026-08-19T07:27:51.571Z</t>
+    <t>2026-08-19T09:09:46.765Z</t>
   </si>
 </sst>
 </file>

</xml_diff>